<commit_message>
Add cache-read token breakdown
</commit_message>
<xml_diff>
--- a/experiments/openwiki-swebench-2026-09/openwiki-swebench-experiment-summary.xlsx
+++ b/experiments/openwiki-swebench-2026-09/openwiki-swebench-experiment-summary.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="实验总表" sheetId="1" r:id="R36c8023f8f864aa8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="证据口径" sheetId="2" r:id="R8dbb424e335a49ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="实验总表" sheetId="1" r:id="R513820a9052c4cd2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="证据口径" sheetId="2" r:id="R7097c65c304d4802"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -276,8 +276,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ExperimentSummary" displayName="ExperimentSummary" ref="A5:AD12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="30">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ExperimentSummary" displayName="ExperimentSummary" ref="A5:AF12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="32">
     <x:tableColumn id="1" name="试验组"/>
     <x:tableColumn id="2" name="模型"/>
     <x:tableColumn id="3" name="OpenWiki介入方式"/>
@@ -299,15 +299,17 @@
     <x:tableColumn id="19" name="平均解题时间(分钟)"/>
     <x:tableColumn id="20" name="相对Baseline耗时变化"/>
     <x:tableColumn id="21" name="平均总token"/>
-    <x:tableColumn id="22" name="最终session总token"/>
-    <x:tableColumn id="23" name="相对Baseline平均token变化"/>
-    <x:tableColumn id="24" name="平均非缓存token"/>
-    <x:tableColumn id="25" name="平均迭代次数"/>
-    <x:tableColumn id="26" name="相对Baseline迭代变化"/>
-    <x:tableColumn id="27" name="Wiki实际返回字节数"/>
-    <x:tableColumn id="28" name="Trace数量"/>
-    <x:tableColumn id="29" name="Wiki注入/使用证据"/>
-    <x:tableColumn id="30" name="可比性说明"/>
+    <x:tableColumn id="22" name="平均缓存读取token"/>
+    <x:tableColumn id="23" name="最终session总token"/>
+    <x:tableColumn id="24" name="最终session缓存读取token"/>
+    <x:tableColumn id="25" name="相对Baseline平均token变化"/>
+    <x:tableColumn id="26" name="平均非缓存token"/>
+    <x:tableColumn id="27" name="平均迭代次数"/>
+    <x:tableColumn id="28" name="相对Baseline迭代变化"/>
+    <x:tableColumn id="29" name="Wiki实际返回字节数"/>
+    <x:tableColumn id="30" name="Trace数量"/>
+    <x:tableColumn id="31" name="Wiki注入/使用证据"/>
+    <x:tableColumn id="32" name="可比性说明"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -529,15 +531,17 @@
     <x:col min="19" max="19" width="15.779999732971191" hidden="0" customWidth="1"/>
     <x:col min="20" max="20" width="17.889999389648438" hidden="0" customWidth="1"/>
     <x:col min="21" max="21" width="11.220000267028809" hidden="0" customWidth="1"/>
-    <x:col min="22" max="22" width="16.780000686645508" hidden="0" customWidth="1"/>
-    <x:col min="23" max="23" width="21.889999389648438" hidden="0" customWidth="1"/>
-    <x:col min="24" max="24" width="14.220000267028809" hidden="0" customWidth="1"/>
-    <x:col min="25" max="25" width="11.779999732971191" hidden="0" customWidth="1"/>
-    <x:col min="26" max="26" width="17.889999389648438" hidden="0" customWidth="1"/>
-    <x:col min="27" max="27" width="16.329999923706055" hidden="0" customWidth="1"/>
-    <x:col min="28" max="28" width="9.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="29" max="29" width="48" hidden="0" customWidth="1"/>
-    <x:col min="30" max="30" width="48" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="15.779999732971191" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="16.780000686645508" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="21.219999313354492" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="21.889999389648438" hidden="0" customWidth="1"/>
+    <x:col min="26" max="26" width="14.220000267028809" hidden="0" customWidth="1"/>
+    <x:col min="27" max="27" width="11.779999732971191" hidden="0" customWidth="1"/>
+    <x:col min="28" max="28" width="17.889999389648438" hidden="0" customWidth="1"/>
+    <x:col min="29" max="29" width="16.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="30" max="30" width="9.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="31" max="31" width="48" hidden="0" customWidth="1"/>
+    <x:col min="32" max="32" width="48" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="2">
@@ -573,6 +577,8 @@
       <x:c r="AB2" s="1"/>
       <x:c r="AC2" s="1"/>
       <x:c r="AD2" s="1"/>
+      <x:c r="AE2" s="1"/>
+      <x:c r="AF2" s="1"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="3" t="str">
@@ -607,6 +613,8 @@
       <x:c r="AB3" s="1"/>
       <x:c r="AC3" s="1"/>
       <x:c r="AD3" s="1"/>
+      <x:c r="AE3" s="1"/>
+      <x:c r="AF3" s="1"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="1"/>
@@ -639,6 +647,8 @@
       <x:c r="AB4" s="1"/>
       <x:c r="AC4" s="1"/>
       <x:c r="AD4" s="1"/>
+      <x:c r="AE4" s="1"/>
+      <x:c r="AF4" s="1"/>
     </x:row>
     <x:row r="5" ht="54" hidden="0" customHeight="1">
       <x:c r="A5" s="15" t="str">
@@ -705,30 +715,36 @@
         <x:v>平均总token</x:v>
       </x:c>
       <x:c r="V5" s="16" t="str">
+        <x:v>平均缓存读取token</x:v>
+      </x:c>
+      <x:c r="W5" s="16" t="str">
         <x:v>最终session总token</x:v>
       </x:c>
-      <x:c r="W5" s="16" t="str">
+      <x:c r="X5" s="16" t="str">
+        <x:v>最终session缓存读取token</x:v>
+      </x:c>
+      <x:c r="Y5" s="16" t="str">
         <x:v>相对Baseline平均token变化</x:v>
       </x:c>
-      <x:c r="X5" s="16" t="str">
+      <x:c r="Z5" s="16" t="str">
         <x:v>平均非缓存token</x:v>
       </x:c>
-      <x:c r="Y5" s="16" t="str">
+      <x:c r="AA5" s="16" t="str">
         <x:v>平均迭代次数</x:v>
       </x:c>
-      <x:c r="Z5" s="16" t="str">
+      <x:c r="AB5" s="16" t="str">
         <x:v>相对Baseline迭代变化</x:v>
       </x:c>
-      <x:c r="AA5" s="16" t="str">
+      <x:c r="AC5" s="16" t="str">
         <x:v>Wiki实际返回字节数</x:v>
       </x:c>
-      <x:c r="AB5" s="16" t="str">
+      <x:c r="AD5" s="16" t="str">
         <x:v>Trace数量</x:v>
       </x:c>
-      <x:c r="AC5" s="16" t="str">
+      <x:c r="AE5" s="16" t="str">
         <x:v>Wiki注入/使用证据</x:v>
       </x:c>
-      <x:c r="AD5" s="17" t="str">
+      <x:c r="AF5" s="17" t="str">
         <x:v>可比性说明</x:v>
       </x:c>
     </x:row>
@@ -797,30 +813,36 @@
         <x:v>3884564.111111111</x:v>
       </x:c>
       <x:c r="V6" s="23" t="n">
+        <x:v>3481560.888888889</x:v>
+      </x:c>
+      <x:c r="W6" s="23" t="n">
         <x:v>69922154</x:v>
       </x:c>
-      <x:c r="W6" s="23" t="n">
-        <x:v>0</x:v>
-      </x:c>
       <x:c r="X6" s="23" t="n">
+        <x:v>62668096</x:v>
+      </x:c>
+      <x:c r="Y6" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Z6" s="23" t="n">
         <x:v>403003.22222222225</x:v>
       </x:c>
-      <x:c r="Y6" s="24" t="n">
+      <x:c r="AA6" s="24" t="n">
         <x:v>65.44444444444444</x:v>
       </x:c>
-      <x:c r="Z6" s="21" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="AA6" s="23" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="AB6" s="23" t="n">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="AC6" s="20" t="str">
+      <x:c r="AB6" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AC6" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AD6" s="23" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="AE6" s="20" t="str">
         <x:v>原始 trace：无 openwiki/*.md 非空内容读取</x:v>
       </x:c>
-      <x:c r="AD6" s="25" t="str">
+      <x:c r="AF6" s="25" t="str">
         <x:v>GLM-5.2 共同18格</x:v>
       </x:c>
     </x:row>
@@ -889,30 +911,36 @@
         <x:v>4277842.222222222</x:v>
       </x:c>
       <x:c r="V7" s="23" t="n">
+        <x:v>3815871.444444444</x:v>
+      </x:c>
+      <x:c r="W7" s="23" t="n">
         <x:v>77001160</x:v>
       </x:c>
-      <x:c r="W7" s="23" t="n">
+      <x:c r="X7" s="23" t="n">
+        <x:v>68685686</x:v>
+      </x:c>
+      <x:c r="Y7" s="21" t="n">
         <x:v>0.10124124608632612</x:v>
       </x:c>
-      <x:c r="X7" s="23" t="n">
+      <x:c r="Z7" s="23" t="n">
         <x:v>461970.77777777775</x:v>
       </x:c>
-      <x:c r="Y7" s="24" t="n">
+      <x:c r="AA7" s="24" t="n">
         <x:v>62.833333333333336</x:v>
       </x:c>
-      <x:c r="Z7" s="21" t="n">
+      <x:c r="AB7" s="21" t="n">
         <x:v>-0.03989813242784379</x:v>
       </x:c>
-      <x:c r="AA7" s="23" t="n">
+      <x:c r="AC7" s="23" t="n">
         <x:v>424993</x:v>
       </x:c>
-      <x:c r="AB7" s="23" t="n">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="AC7" s="20" t="str">
+      <x:c r="AD7" s="23" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="AE7" s="20" t="str">
         <x:v>原始 trace：18/18 有效读取，且均早于首次源码编辑</x:v>
       </x:c>
-      <x:c r="AD7" s="25" t="str">
+      <x:c r="AF7" s="25" t="str">
         <x:v>GLM-5.2 共同18格</x:v>
       </x:c>
     </x:row>
@@ -981,30 +1009,36 @@
         <x:v>5007742.777777778</x:v>
       </x:c>
       <x:c r="V8" s="23" t="n">
+        <x:v>4378404.055555556</x:v>
+      </x:c>
+      <x:c r="W8" s="23" t="n">
         <x:v>90139370</x:v>
       </x:c>
-      <x:c r="W8" s="23" t="n">
+      <x:c r="X8" s="23" t="n">
+        <x:v>78811273</x:v>
+      </x:c>
+      <x:c r="Y8" s="21" t="n">
         <x:v>0.28913891868949015</x:v>
       </x:c>
-      <x:c r="X8" s="23" t="n">
+      <x:c r="Z8" s="23" t="n">
         <x:v>629338.7222222222</x:v>
       </x:c>
-      <x:c r="Y8" s="24" t="n">
+      <x:c r="AA8" s="24" t="n">
         <x:v>65.72222222222223</x:v>
       </x:c>
-      <x:c r="Z8" s="21" t="n">
+      <x:c r="AB8" s="21" t="n">
         <x:v>0.004244482173175079</x:v>
       </x:c>
-      <x:c r="AA8" s="23" t="n">
+      <x:c r="AC8" s="23" t="n">
         <x:v>10104</x:v>
       </x:c>
-      <x:c r="AB8" s="23" t="n">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="AC8" s="20" t="str">
+      <x:c r="AD8" s="23" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="AE8" s="20" t="str">
         <x:v>原始 trace：5/18 有效读取；2/18 早于首次源码编辑</x:v>
       </x:c>
-      <x:c r="AD8" s="25" t="str">
+      <x:c r="AF8" s="25" t="str">
         <x:v>GLM-5.2 共同18格</x:v>
       </x:c>
     </x:row>
@@ -1073,30 +1107,36 @@
         <x:v>4757041.833333333</x:v>
       </x:c>
       <x:c r="V9" s="23" t="n">
+        <x:v>4113711.7777777775</x:v>
+      </x:c>
+      <x:c r="W9" s="23" t="n">
         <x:v>85626753</x:v>
       </x:c>
-      <x:c r="W9" s="23" t="n">
+      <x:c r="X9" s="23" t="n">
+        <x:v>74046812</x:v>
+      </x:c>
+      <x:c r="Y9" s="21" t="n">
         <x:v>0.2246011900605922</x:v>
       </x:c>
-      <x:c r="X9" s="23" t="n">
+      <x:c r="Z9" s="23" t="n">
         <x:v>643330.0555555555</x:v>
       </x:c>
-      <x:c r="Y9" s="24" t="n">
+      <x:c r="AA9" s="24" t="n">
         <x:v>70.11111111111111</x:v>
       </x:c>
-      <x:c r="Z9" s="21" t="n">
+      <x:c r="AB9" s="21" t="n">
         <x:v>0.07130730050933787</x:v>
       </x:c>
-      <x:c r="AA9" s="23" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="AB9" s="23" t="n">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="AC9" s="20" t="str">
+      <x:c r="AC9" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AD9" s="23" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="AE9" s="20" t="str">
         <x:v>runner 注入与卡片哈希校验18/18；solver主动Wiki读取0/18</x:v>
       </x:c>
-      <x:c r="AD9" s="25" t="str">
+      <x:c r="AF9" s="25" t="str">
         <x:v>GLM-5.2 共同18格</x:v>
       </x:c>
     </x:row>
@@ -1165,30 +1205,36 @@
         <x:v>3883684.388888889</x:v>
       </x:c>
       <x:c r="V10" s="23" t="n">
+        <x:v>3504565.3333333335</x:v>
+      </x:c>
+      <x:c r="W10" s="23" t="n">
         <x:v>69906319</x:v>
       </x:c>
-      <x:c r="W10" s="23" t="n">
+      <x:c r="X10" s="23" t="n">
+        <x:v>63082176</x:v>
+      </x:c>
+      <x:c r="Y10" s="21" t="n">
         <x:v>-0.00022646613546828398</x:v>
       </x:c>
-      <x:c r="X10" s="23" t="n">
+      <x:c r="Z10" s="23" t="n">
         <x:v>379119.05555555556</x:v>
       </x:c>
-      <x:c r="Y10" s="24" t="n">
+      <x:c r="AA10" s="24" t="n">
         <x:v>66.83333333333333</x:v>
       </x:c>
-      <x:c r="Z10" s="21" t="n">
+      <x:c r="AB10" s="21" t="n">
         <x:v>0.021222410865874286</x:v>
       </x:c>
-      <x:c r="AA10" s="23" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="AB10" s="23" t="n">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="AC10" s="20" t="str">
+      <x:c r="AC10" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AD10" s="23" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="AE10" s="20" t="str">
         <x:v>原始 trace：有效 Wiki 内容读取0/18；(no output)不计调用</x:v>
       </x:c>
-      <x:c r="AD10" s="25" t="str">
+      <x:c r="AF10" s="25" t="str">
         <x:v>GLM-5.2 共同18格</x:v>
       </x:c>
     </x:row>
@@ -1253,26 +1299,32 @@
         <x:v>6886967.823529412</x:v>
       </x:c>
       <x:c r="V11" s="23" t="n">
+        <x:v>6053078.588235294</x:v>
+      </x:c>
+      <x:c r="W11" s="23" t="n">
         <x:v>117078453</x:v>
       </x:c>
-      <x:c r="W11" s="23"/>
       <x:c r="X11" s="23" t="n">
+        <x:v>102902336</x:v>
+      </x:c>
+      <x:c r="Y11" s="21"/>
+      <x:c r="Z11" s="23" t="n">
         <x:v>833889.2352941176</x:v>
       </x:c>
-      <x:c r="Y11" s="24" t="n">
+      <x:c r="AA11" s="24" t="n">
         <x:v>71.6470588235294</x:v>
       </x:c>
-      <x:c r="Z11" s="21"/>
-      <x:c r="AA11" s="23" t="n">
+      <x:c r="AB11" s="21"/>
+      <x:c r="AC11" s="23" t="n">
         <x:v>428043</x:v>
       </x:c>
-      <x:c r="AB11" s="23" t="n">
+      <x:c r="AD11" s="23" t="n">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="AC11" s="20" t="str">
+      <x:c r="AE11" s="20" t="str">
         <x:v>原始 trace：已评分17格均读取index和quickstart，且早于首次编辑</x:v>
       </x:c>
-      <x:c r="AD11" s="25" t="str">
+      <x:c r="AF11" s="25" t="str">
         <x:v>仅17格官方结果，不与18格组直接比较</x:v>
       </x:c>
     </x:row>
@@ -1337,37 +1389,43 @@
         <x:v>5525577.055555556</x:v>
       </x:c>
       <x:c r="V12" s="31" t="n">
+        <x:v>5297927.111111112</x:v>
+      </x:c>
+      <x:c r="W12" s="31" t="n">
         <x:v>99460387</x:v>
       </x:c>
-      <x:c r="W12" s="31"/>
       <x:c r="X12" s="31" t="n">
+        <x:v>95362688</x:v>
+      </x:c>
+      <x:c r="Y12" s="29"/>
+      <x:c r="Z12" s="31" t="n">
         <x:v>227649.94444444444</x:v>
       </x:c>
-      <x:c r="Y12" s="32" t="n">
+      <x:c r="AA12" s="32" t="n">
         <x:v>61.5</x:v>
       </x:c>
-      <x:c r="Z12" s="29"/>
-      <x:c r="AA12" s="31" t="n">
+      <x:c r="AB12" s="29"/>
+      <x:c r="AC12" s="31" t="n">
         <x:v>449049</x:v>
       </x:c>
-      <x:c r="AB12" s="31" t="n">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="AC12" s="28" t="str">
+      <x:c r="AD12" s="31" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="AE12" s="28" t="str">
         <x:v>原始 trace：18/18有效读取；16/18早于首次编辑；严格协议7/18</x:v>
       </x:c>
-      <x:c r="AD12" s="33" t="str">
+      <x:c r="AF12" s="33" t="str">
         <x:v>模型不同；11/18协议无效，不作跨模型因果比较</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A2:AD2"/>
-    <x:mergeCell ref="A3:AD3"/>
+    <x:mergeCell ref="A2:AF2"/>
+    <x:mergeCell ref="A3:AF3"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R801eee165f704ea5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd35f05e504a34993"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1433,30 +1491,38 @@
         <x:v>总token</x:v>
       </x:c>
       <x:c r="B8" s="41" t="str">
-        <x:v>含缓存读取；非缓存token为input+output+reasoning。均不含OpenWiki建库和Harness。</x:v>
+        <x:v>来自每个step-finish的tokens.total；总token = input + output + reasoning + cache.read。本表同时列平均值与最终入表session合计。</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="37" t="str">
-        <x:v>重试成本</x:v>
+        <x:v>缓存读取</x:v>
       </x:c>
       <x:c r="B9" s="41" t="str">
-        <x:v>表中均值只计最终入表session。GLM-5.3组43个solver attempt总计273,506,098 total tokens。</x:v>
+        <x:v>直接累加每个step-finish的part.tokens.cache.read。125条入表trace逐条验证等于total减去input、output、reasoning。</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="37" t="str">
+        <x:v>重试成本</x:v>
+      </x:c>
+      <x:c r="B10" s="41" t="str">
+        <x:v>表中均值只计最终入表session。GLM-5.3组43个solver attempt总计273,506,098 total tokens。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
+      <x:c r="A11" s="37" t="str">
         <x:v>可比性</x:v>
       </x:c>
-      <x:c r="B10" s="41" t="str">
+      <x:c r="B11" s="41" t="str">
         <x:v>GLM-5.3组模型和协议成功率均不同，不能与GLM-5.2分差作因果比较。</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="15" hidden="0" customHeight="1">
-      <x:c r="A11" s="39" t="str">
+    <x:row r="12" ht="15" hidden="0" customHeight="1">
+      <x:c r="A12" s="39" t="str">
         <x:v>原始审计</x:v>
       </x:c>
-      <x:c r="B11" s="42" t="str">
+      <x:c r="B12" s="42" t="str">
         <x:v>/home/zhangzijian/openwiki-swebench/results/openwiki-all-experiments-2026-09-22.jsonl（920）</x:v>
       </x:c>
     </x:row>

</xml_diff>